<commit_message>
update perawatan dari web
</commit_message>
<xml_diff>
--- a/data/Rekakapitulasi-Perawatan.xlsx
+++ b/data/Rekakapitulasi-Perawatan.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\3. TSSP.3\1. Laporan Bulanan\2026\4. Apr\KP\Perawatan Peralatan\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67D40EBF-A6B0-45C9-B791-9855C029C96D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A328FFF-B586-4581-9D38-A696B5DE5C47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{89E2D6B6-1DCD-4189-A113-A83F3B882A03}"/>
   </bookViews>
   <sheets>
     <sheet name="Perawatan" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Perawatan!$A$1:$J$392</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -12335,6 +12338,7 @@
       <c r="J392" s="1"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:J392" xr:uid="{045E82A1-AFA5-46B1-A9F4-12F5B515B637}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>